<commit_message>
fix search and events
</commit_message>
<xml_diff>
--- a/public/fortal_consolidado.xlsx
+++ b/public/fortal_consolidado.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="234">
   <si>
     <t>name</t>
   </si>
@@ -178,15 +178,6 @@
     <t>CENTRO DE CONVENÇÕES E EXPOSIÇÕES INDEPENDENTES</t>
   </si>
   <si>
-    <t>176.899m²</t>
-  </si>
-  <si>
-    <t>13.500m²</t>
-  </si>
-  <si>
-    <t>14m²</t>
-  </si>
-  <si>
     <t>2 pavilhoes de 13.500m²</t>
   </si>
   <si>
@@ -194,9 +185,6 @@
   </si>
   <si>
     <t>100m²</t>
-  </si>
-  <si>
-    <t>18 salas</t>
   </si>
   <si>
     <t>NENHUM</t>
@@ -333,9 +321,6 @@
     <t>PESSOA COM DEFICIÊNCIA FÍSICA / BAIXA ESTATURA, PESSOA COM DEFICIÊNCIA FÍSICA / CADEIRANTE</t>
   </si>
   <si>
-    <t>2081m²</t>
-  </si>
-  <si>
     <t>SONORIZAÇÃO, EQUIPAMENTOS AUDIOVISUAIS, INTERNET WIRELESS, ALIMENTAÇÃO, RECURSOS HUMANOS</t>
   </si>
   <si>
@@ -411,9 +396,6 @@
   </si>
   <si>
     <t>128M²</t>
-  </si>
-  <si>
-    <t>3,70M</t>
   </si>
   <si>
     <t>9M²</t>
@@ -952,7 +934,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -978,6 +960,12 @@
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
     <xf borderId="3" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
@@ -1000,6 +988,9 @@
     </xf>
     <xf borderId="3" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1512,212 +1503,212 @@
       <c r="AB2" s="8"/>
       <c r="AC2" s="8"/>
       <c r="AD2" s="8"/>
-      <c r="AE2" s="5" t="s">
+      <c r="AE2" s="9">
+        <v>176899.0</v>
+      </c>
+      <c r="AF2" s="9">
+        <v>13500.0</v>
+      </c>
+      <c r="AG2" s="10">
+        <v>14.0</v>
+      </c>
+      <c r="AH2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AF2" s="5" t="s">
+      <c r="AI2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AG2" s="5" t="s">
+      <c r="AJ2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="AH2" s="5" t="s">
+      <c r="AK2" s="10">
+        <v>18.0</v>
+      </c>
+      <c r="AL2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="AI2" s="5" t="s">
+      <c r="AM2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="AJ2" s="5" t="s">
+      <c r="AN2" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="AK2" s="5" t="s">
+      <c r="AO2" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="AL2" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AM2" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AN2" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AO2" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="AP2" s="8"/>
       <c r="AQ2" s="8"/>
       <c r="AR2" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="AS2" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT2" s="9"/>
-      <c r="AU2" s="10"/>
-      <c r="AV2" s="10"/>
-      <c r="AW2" s="10"/>
-      <c r="AX2" s="10"/>
-      <c r="AY2" s="10"/>
-      <c r="AZ2" s="10"/>
+        <v>63</v>
+      </c>
+      <c r="AT2" s="11"/>
+      <c r="AU2" s="12"/>
+      <c r="AV2" s="12"/>
+      <c r="AW2" s="12"/>
+      <c r="AX2" s="12"/>
+      <c r="AY2" s="12"/>
+      <c r="AZ2" s="12"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="15">
+        <v>8.5988143785E10</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="G3" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="H3" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="13">
+      <c r="I3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="M3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="N3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="O3" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="P3" s="15">
+        <v>8.534661922E9</v>
+      </c>
+      <c r="Q3" s="15">
         <v>8.5988143785E10</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" s="14" t="s">
+      <c r="R3" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="T3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="J3" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="M3" s="12" t="s">
+      <c r="U3" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="N3" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="O3" s="12" t="s">
+      <c r="V3" s="17"/>
+      <c r="W3" s="17"/>
+      <c r="X3" s="17"/>
+      <c r="Y3" s="17"/>
+      <c r="Z3" s="17"/>
+      <c r="AA3" s="17"/>
+      <c r="AB3" s="17"/>
+      <c r="AC3" s="17"/>
+      <c r="AD3" s="17"/>
+      <c r="AE3" s="17"/>
+      <c r="AF3" s="17"/>
+      <c r="AG3" s="17"/>
+      <c r="AH3" s="17"/>
+      <c r="AI3" s="17"/>
+      <c r="AJ3" s="17"/>
+      <c r="AK3" s="17"/>
+      <c r="AL3" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="P3" s="13">
-        <v>8.534661922E9</v>
-      </c>
-      <c r="Q3" s="13">
-        <v>8.5988143785E10</v>
-      </c>
-      <c r="R3" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="S3" s="12" t="s">
+      <c r="AM3" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="AN3" s="17"/>
+      <c r="AO3" s="17"/>
+      <c r="AP3" s="17"/>
+      <c r="AQ3" s="17"/>
+      <c r="AR3" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="AS3" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="V3" s="15"/>
-      <c r="W3" s="15"/>
-      <c r="X3" s="15"/>
-      <c r="Y3" s="15"/>
-      <c r="Z3" s="15"/>
-      <c r="AA3" s="15"/>
-      <c r="AB3" s="15"/>
-      <c r="AC3" s="15"/>
-      <c r="AD3" s="15"/>
-      <c r="AE3" s="15"/>
-      <c r="AF3" s="15"/>
-      <c r="AG3" s="15"/>
-      <c r="AH3" s="15"/>
-      <c r="AI3" s="15"/>
-      <c r="AJ3" s="15"/>
-      <c r="AK3" s="15"/>
-      <c r="AL3" s="12" t="s">
+      <c r="AT3" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="AM3" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN3" s="15"/>
-      <c r="AO3" s="15"/>
-      <c r="AP3" s="15"/>
-      <c r="AQ3" s="15"/>
-      <c r="AR3" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="AS3" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT3" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="AU3" s="10"/>
-      <c r="AV3" s="10"/>
-      <c r="AW3" s="10"/>
-      <c r="AX3" s="10"/>
-      <c r="AY3" s="10"/>
-      <c r="AZ3" s="10"/>
+      <c r="AU3" s="12"/>
+      <c r="AV3" s="12"/>
+      <c r="AW3" s="12"/>
+      <c r="AX3" s="12"/>
+      <c r="AY3" s="12"/>
+      <c r="AZ3" s="12"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="F4" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="G4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="H4" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="J4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="P4" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="Q4" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>51</v>
@@ -1726,10 +1717,10 @@
         <v>52</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="V4" s="6">
         <v>270.0</v>
@@ -1738,28 +1729,28 @@
         <v>530.0</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="AA4" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="AC4" s="6">
         <v>14.0</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="AE4" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
+      </c>
+      <c r="AE4" s="10">
+        <v>2081.0</v>
       </c>
       <c r="AF4" s="6">
         <v>1000.0</v>
@@ -1780,224 +1771,224 @@
         <v>15.0</v>
       </c>
       <c r="AL4" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="AM4" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="AN4" s="6">
         <v>180.0</v>
       </c>
       <c r="AO4" s="5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="AP4" s="5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="AQ4" s="5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="AR4" s="5" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="AS4" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT4" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="AU4" s="10"/>
-      <c r="AV4" s="10"/>
-      <c r="AW4" s="10"/>
-      <c r="AX4" s="10"/>
-      <c r="AY4" s="10"/>
-      <c r="AZ4" s="10"/>
+        <v>80</v>
+      </c>
+      <c r="AT4" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="AU4" s="12"/>
+      <c r="AV4" s="12"/>
+      <c r="AW4" s="12"/>
+      <c r="AX4" s="12"/>
+      <c r="AY4" s="12"/>
+      <c r="AZ4" s="12"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="15">
+        <v>8.5988276395E10</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="H5" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="I5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="N5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="O5" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="13">
-        <v>8.5988276395E10</v>
-      </c>
-      <c r="E5" s="12" t="s">
+      <c r="P5" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="Q5" s="17"/>
+      <c r="R5" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="S5" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="T5" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="U5" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="V5" s="15">
+        <v>273.0</v>
+      </c>
+      <c r="W5" s="15">
+        <v>273.0</v>
+      </c>
+      <c r="X5" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y5" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="N5" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="O5" s="12" t="s">
+      <c r="Z5" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="P5" s="12" t="s">
+      <c r="AA5" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="S5" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="T5" s="12" t="s">
+      <c r="AB5" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC5" s="15">
+        <v>8.0</v>
+      </c>
+      <c r="AD5" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="U5" s="12" t="s">
+      <c r="AE5" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="V5" s="13">
-        <v>273.0</v>
-      </c>
-      <c r="W5" s="13">
-        <v>273.0</v>
-      </c>
-      <c r="X5" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y5" s="12" t="s">
+      <c r="AF5" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="Z5" s="12" t="s">
+      <c r="AG5" s="20">
+        <v>3.7</v>
+      </c>
+      <c r="AH5" s="17"/>
+      <c r="AI5" s="17"/>
+      <c r="AJ5" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="AA5" s="12" t="s">
+      <c r="AK5" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="AL5" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="AB5" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC5" s="13">
-        <v>8.0</v>
-      </c>
-      <c r="AD5" s="12" t="s">
+      <c r="AM5" s="17"/>
+      <c r="AN5" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="AE5" s="12" t="s">
+      <c r="AO5" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="AF5" s="12" t="s">
+      <c r="AP5" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="AG5" s="12" t="s">
+      <c r="AQ5" s="17"/>
+      <c r="AR5" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="AH5" s="15"/>
-      <c r="AI5" s="15"/>
-      <c r="AJ5" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="AK5" s="13">
-        <v>6.0</v>
-      </c>
-      <c r="AL5" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="AM5" s="15"/>
-      <c r="AN5" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="AO5" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="AP5" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="AQ5" s="15"/>
-      <c r="AR5" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="AS5" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT5" s="18"/>
-      <c r="AU5" s="10"/>
-      <c r="AV5" s="10"/>
-      <c r="AW5" s="10"/>
-      <c r="AX5" s="10"/>
-      <c r="AY5" s="10"/>
-      <c r="AZ5" s="10"/>
+      <c r="AS5" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT5" s="21"/>
+      <c r="AU5" s="12"/>
+      <c r="AV5" s="12"/>
+      <c r="AW5" s="12"/>
+      <c r="AX5" s="12"/>
+      <c r="AY5" s="12"/>
+      <c r="AZ5" s="12"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="H6" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="I6" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="K6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="N6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="P6" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="Q6" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>150</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>51</v>
@@ -2006,10 +1997,10 @@
         <v>52</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="V6" s="6">
         <v>200.0</v>
@@ -2018,25 +2009,25 @@
         <v>426.0</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="AC6" s="6">
         <v>5.0</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="AE6" s="8"/>
       <c r="AF6" s="6">
@@ -2048,222 +2039,222 @@
       <c r="AH6" s="8"/>
       <c r="AI6" s="8"/>
       <c r="AJ6" s="5" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="AK6" s="6">
         <v>8.0</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="AM6" s="5" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="AN6" s="5" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="AO6" s="5" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="AP6" s="8"/>
       <c r="AQ6" s="5" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="AR6" s="5" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="AS6" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT6" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="AU6" s="10"/>
-      <c r="AV6" s="10"/>
-      <c r="AW6" s="10"/>
-      <c r="AX6" s="10"/>
-      <c r="AY6" s="10"/>
-      <c r="AZ6" s="10"/>
+        <v>80</v>
+      </c>
+      <c r="AT6" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="AU6" s="12"/>
+      <c r="AV6" s="12"/>
+      <c r="AW6" s="12"/>
+      <c r="AX6" s="12"/>
+      <c r="AY6" s="12"/>
+      <c r="AZ6" s="12"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="I7" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="J7" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="M7" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="N7" s="17"/>
+      <c r="O7" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="P7" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="Q7" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="G7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="H7" s="14" t="s">
+      <c r="R7" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="S7" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="T7" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="U7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="V7" s="15">
+        <v>230.0</v>
+      </c>
+      <c r="W7" s="15">
+        <v>339.0</v>
+      </c>
+      <c r="X7" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y7" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z7" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="J7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="M7" s="14" t="s">
+      <c r="AA7" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="N7" s="15"/>
-      <c r="O7" s="12" t="s">
+      <c r="AB7" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC7" s="15">
+        <v>3.0</v>
+      </c>
+      <c r="AD7" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE7" s="15">
+        <v>1755.0</v>
+      </c>
+      <c r="AF7" s="15">
+        <v>855.0</v>
+      </c>
+      <c r="AG7" s="15">
+        <v>2.73</v>
+      </c>
+      <c r="AH7" s="17"/>
+      <c r="AI7" s="17"/>
+      <c r="AJ7" s="15">
+        <v>45.0</v>
+      </c>
+      <c r="AK7" s="15">
+        <v>16.0</v>
+      </c>
+      <c r="AL7" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="AM7" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AN7" s="15">
+        <v>150.0</v>
+      </c>
+      <c r="AO7" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="AP7" s="17"/>
+      <c r="AQ7" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="AR7" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="R7" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="S7" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="T7" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="U7" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="V7" s="13">
-        <v>230.0</v>
-      </c>
-      <c r="W7" s="13">
-        <v>339.0</v>
-      </c>
-      <c r="X7" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y7" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="Z7" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA7" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="AB7" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC7" s="13">
-        <v>3.0</v>
-      </c>
-      <c r="AD7" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="AE7" s="13">
-        <v>1755.0</v>
-      </c>
-      <c r="AF7" s="13">
-        <v>855.0</v>
-      </c>
-      <c r="AG7" s="13">
-        <v>2.73</v>
-      </c>
-      <c r="AH7" s="15"/>
-      <c r="AI7" s="15"/>
-      <c r="AJ7" s="13">
-        <v>45.0</v>
-      </c>
-      <c r="AK7" s="13">
-        <v>16.0</v>
-      </c>
-      <c r="AL7" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM7" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN7" s="13">
-        <v>150.0</v>
-      </c>
-      <c r="AO7" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="AP7" s="15"/>
-      <c r="AQ7" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="AR7" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="AS7" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT7" s="18"/>
-      <c r="AU7" s="10"/>
-      <c r="AV7" s="10"/>
-      <c r="AW7" s="10"/>
-      <c r="AX7" s="10"/>
-      <c r="AY7" s="10"/>
-      <c r="AZ7" s="10"/>
+      <c r="AS7" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AT7" s="21"/>
+      <c r="AU7" s="12"/>
+      <c r="AV7" s="12"/>
+      <c r="AW7" s="12"/>
+      <c r="AX7" s="12"/>
+      <c r="AY7" s="12"/>
+      <c r="AZ7" s="12"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D8" s="6">
         <v>8.5982080161E10</v>
       </c>
       <c r="E8" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="K8" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="L8" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="M8" s="7" t="s">
         <v>187</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>193</v>
       </c>
       <c r="N8" s="8"/>
       <c r="O8" s="5" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="P8" s="6">
         <v>7.140404999E9</v>
@@ -2278,10 +2269,10 @@
         <v>52</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="V8" s="6">
         <v>300.0</v>
@@ -2290,25 +2281,25 @@
         <v>300.0</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="AA8" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="AC8" s="6">
         <v>8.0</v>
       </c>
       <c r="AD8" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="AE8" s="6">
         <v>1300.0</v>
@@ -2328,82 +2319,82 @@
         <v>8.0</v>
       </c>
       <c r="AL8" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="AM8" s="5" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="AN8" s="6">
         <v>700.0</v>
       </c>
       <c r="AO8" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="AP8" s="8"/>
       <c r="AQ8" s="8"/>
       <c r="AR8" s="8"/>
       <c r="AS8" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT8" s="9"/>
-      <c r="AU8" s="10"/>
-      <c r="AV8" s="10"/>
-      <c r="AW8" s="10"/>
-      <c r="AX8" s="10"/>
-      <c r="AY8" s="10"/>
-      <c r="AZ8" s="10"/>
+        <v>63</v>
+      </c>
+      <c r="AT8" s="11"/>
+      <c r="AU8" s="12"/>
+      <c r="AV8" s="12"/>
+      <c r="AW8" s="12"/>
+      <c r="AX8" s="12"/>
+      <c r="AY8" s="12"/>
+      <c r="AZ8" s="12"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="I9" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="J9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="M9" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="N9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="O9" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="P9" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="Q9" s="5" t="s">
         <v>206</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="N9" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>212</v>
       </c>
       <c r="R9" s="5" t="s">
         <v>51</v>
@@ -2412,10 +2403,10 @@
         <v>52</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="V9" s="6">
         <v>192.0</v>
@@ -2424,25 +2415,25 @@
         <v>432.0</v>
       </c>
       <c r="X9" s="5" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="Y9" s="5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="AC9" s="6">
         <v>4.0</v>
       </c>
       <c r="AD9" s="5" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="AE9" s="6">
         <v>3800.0</v>
@@ -2466,154 +2457,154 @@
         <v>14.0</v>
       </c>
       <c r="AL9" s="5" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="AM9" s="5" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="AN9" s="5" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="AO9" s="8"/>
       <c r="AP9" s="8"/>
       <c r="AQ9" s="5" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="AR9" s="5" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="AS9" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT9" s="9"/>
-      <c r="AU9" s="10"/>
-      <c r="AV9" s="10"/>
-      <c r="AW9" s="10"/>
-      <c r="AX9" s="10"/>
-      <c r="AY9" s="10"/>
-      <c r="AZ9" s="10"/>
+        <v>63</v>
+      </c>
+      <c r="AT9" s="11"/>
+      <c r="AU9" s="12"/>
+      <c r="AV9" s="12"/>
+      <c r="AW9" s="12"/>
+      <c r="AX9" s="12"/>
+      <c r="AY9" s="12"/>
+      <c r="AZ9" s="12"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>220</v>
+      </c>
+      <c r="H10" s="25" t="s">
         <v>221</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="21" t="s">
+      <c r="I10" s="25" t="s">
         <v>222</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="J10" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="K10" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="L10" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="M10" s="25" t="s">
         <v>225</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="N10" s="23"/>
+      <c r="O10" s="24" t="s">
         <v>226</v>
       </c>
-      <c r="H10" s="22" t="s">
+      <c r="P10" s="24" t="s">
         <v>227</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="Q10" s="24" t="s">
+        <v>227</v>
+      </c>
+      <c r="R10" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="S10" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="T10" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="J10" s="22" t="s">
+      <c r="U10" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="V10" s="26">
+        <v>98.0</v>
+      </c>
+      <c r="W10" s="26">
+        <v>214.0</v>
+      </c>
+      <c r="X10" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y10" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z10" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="AA10" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="K10" s="22" t="s">
+      <c r="AB10" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC10" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="AD10" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="AE10" s="23"/>
+      <c r="AF10" s="23"/>
+      <c r="AG10" s="23"/>
+      <c r="AH10" s="23"/>
+      <c r="AI10" s="23"/>
+      <c r="AJ10" s="23"/>
+      <c r="AK10" s="26">
+        <v>4.0</v>
+      </c>
+      <c r="AL10" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="L10" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="M10" s="22" t="s">
+      <c r="AM10" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="N10" s="20"/>
-      <c r="O10" s="21" t="s">
+      <c r="AN10" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="P10" s="21" t="s">
+      <c r="AO10" s="23"/>
+      <c r="AP10" s="23"/>
+      <c r="AQ10" s="23"/>
+      <c r="AR10" s="24" t="s">
         <v>233</v>
       </c>
-      <c r="Q10" s="21" t="s">
-        <v>233</v>
-      </c>
-      <c r="R10" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="S10" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="T10" s="21" t="s">
-        <v>234</v>
-      </c>
-      <c r="U10" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="V10" s="23">
-        <v>98.0</v>
-      </c>
-      <c r="W10" s="23">
-        <v>214.0</v>
-      </c>
-      <c r="X10" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y10" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="Z10" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="AA10" s="21" t="s">
-        <v>235</v>
-      </c>
-      <c r="AB10" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC10" s="23">
-        <v>2.0</v>
-      </c>
-      <c r="AD10" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="AE10" s="20"/>
-      <c r="AF10" s="20"/>
-      <c r="AG10" s="20"/>
-      <c r="AH10" s="20"/>
-      <c r="AI10" s="20"/>
-      <c r="AJ10" s="20"/>
-      <c r="AK10" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="AL10" s="21" t="s">
-        <v>236</v>
-      </c>
-      <c r="AM10" s="21" t="s">
-        <v>237</v>
-      </c>
-      <c r="AN10" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="AO10" s="20"/>
-      <c r="AP10" s="20"/>
-      <c r="AQ10" s="20"/>
-      <c r="AR10" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="AS10" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT10" s="24"/>
-      <c r="AU10" s="10"/>
-      <c r="AV10" s="10"/>
-      <c r="AW10" s="10"/>
-      <c r="AX10" s="10"/>
-      <c r="AY10" s="10"/>
-      <c r="AZ10" s="10"/>
+      <c r="AS10" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT10" s="27"/>
+      <c r="AU10" s="12"/>
+      <c r="AV10" s="12"/>
+      <c r="AW10" s="12"/>
+      <c r="AX10" s="12"/>
+      <c r="AY10" s="12"/>
+      <c r="AZ10" s="12"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>